<commit_message>
Added BLEU, ROUGE-1 F and ROUGE-L F
</commit_message>
<xml_diff>
--- a/demo/ic_demo.xlsx
+++ b/demo/ic_demo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\o.hamed\Documents\Dev\GitHub\image-captioning\demo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\v.patil\Documents\Dev\Github\image-captioning\demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2A4EAB-B2C0-4B79-8009-BBBA4BB41D74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6740AA00-D0BF-4AF3-866B-4EC35D0918EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29895" yWindow="8490" windowWidth="38220" windowHeight="17550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -537,13 +537,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E20"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.28515625" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
-    <col min="4" max="4" width="161.85546875" customWidth="1"/>
-    <col min="5" max="5" width="157.140625" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" customWidth="1"/>
+    <col min="4" max="4" width="161.88671875" customWidth="1"/>
+    <col min="5" max="5" width="157.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">

</xml_diff>